<commit_message>
Phase 4: Benchmark date-coherence, ground-truth validation guard, location-aware matching & ambiguity recalibration
</commit_message>
<xml_diff>
--- a/data/synthetic_field_updates.xlsx
+++ b/data/synthetic_field_updates.xlsx
@@ -466,7 +466,7 @@
       </c>
       <c r="B2" t="inlineStr">
         <is>
-          <t>2026-04-16</t>
+          <t>2026-06-19</t>
         </is>
       </c>
       <c r="C2" t="inlineStr">
@@ -508,7 +508,7 @@
       </c>
       <c r="B3" t="inlineStr">
         <is>
-          <t>2026-04-17</t>
+          <t>2026-05-09</t>
         </is>
       </c>
       <c r="C3" t="inlineStr">
@@ -550,7 +550,7 @@
       </c>
       <c r="B4" t="inlineStr">
         <is>
-          <t>2026-04-18</t>
+          <t>2026-06-22</t>
         </is>
       </c>
       <c r="C4" t="inlineStr">
@@ -592,7 +592,7 @@
       </c>
       <c r="B5" t="inlineStr">
         <is>
-          <t>2026-04-19</t>
+          <t>2026-07-09</t>
         </is>
       </c>
       <c r="C5" t="inlineStr">
@@ -634,7 +634,7 @@
       </c>
       <c r="B6" t="inlineStr">
         <is>
-          <t>2026-04-20</t>
+          <t>2026-04-29</t>
         </is>
       </c>
       <c r="C6" t="inlineStr">
@@ -676,7 +676,7 @@
       </c>
       <c r="B7" t="inlineStr">
         <is>
-          <t>2026-04-21</t>
+          <t>2026-07-10</t>
         </is>
       </c>
       <c r="C7" t="inlineStr">
@@ -718,7 +718,7 @@
       </c>
       <c r="B8" t="inlineStr">
         <is>
-          <t>2026-04-22</t>
+          <t>2026-05-15</t>
         </is>
       </c>
       <c r="C8" t="inlineStr">
@@ -760,7 +760,7 @@
       </c>
       <c r="B9" t="inlineStr">
         <is>
-          <t>2026-04-23</t>
+          <t>2026-07-23</t>
         </is>
       </c>
       <c r="C9" t="inlineStr">
@@ -802,7 +802,7 @@
       </c>
       <c r="B10" t="inlineStr">
         <is>
-          <t>2026-04-24</t>
+          <t>2026-06-15</t>
         </is>
       </c>
       <c r="C10" t="inlineStr">
@@ -844,7 +844,7 @@
       </c>
       <c r="B11" t="inlineStr">
         <is>
-          <t>2026-04-25</t>
+          <t>2026-06-09</t>
         </is>
       </c>
       <c r="C11" t="inlineStr">
@@ -886,7 +886,7 @@
       </c>
       <c r="B12" t="inlineStr">
         <is>
-          <t>2026-04-26</t>
+          <t>2026-09-06</t>
         </is>
       </c>
       <c r="C12" t="inlineStr">
@@ -928,7 +928,7 @@
       </c>
       <c r="B13" t="inlineStr">
         <is>
-          <t>2026-04-27</t>
+          <t>2026-08-29</t>
         </is>
       </c>
       <c r="C13" t="inlineStr">
@@ -970,7 +970,7 @@
       </c>
       <c r="B14" t="inlineStr">
         <is>
-          <t>2026-04-28</t>
+          <t>2026-06-28</t>
         </is>
       </c>
       <c r="C14" t="inlineStr">
@@ -1012,7 +1012,7 @@
       </c>
       <c r="B15" t="inlineStr">
         <is>
-          <t>2026-04-29</t>
+          <t>2026-07-29</t>
         </is>
       </c>
       <c r="C15" t="inlineStr">
@@ -1054,7 +1054,7 @@
       </c>
       <c r="B16" t="inlineStr">
         <is>
-          <t>2026-04-30</t>
+          <t>2026-05-17</t>
         </is>
       </c>
       <c r="C16" t="inlineStr">
@@ -1096,7 +1096,7 @@
       </c>
       <c r="B17" t="inlineStr">
         <is>
-          <t>2026-05-01</t>
+          <t>2026-07-14</t>
         </is>
       </c>
       <c r="C17" t="inlineStr">
@@ -1138,7 +1138,7 @@
       </c>
       <c r="B18" t="inlineStr">
         <is>
-          <t>2026-05-02</t>
+          <t>2026-08-12</t>
         </is>
       </c>
       <c r="C18" t="inlineStr">
@@ -1180,7 +1180,7 @@
       </c>
       <c r="B19" t="inlineStr">
         <is>
-          <t>2026-05-03</t>
+          <t>2026-06-25</t>
         </is>
       </c>
       <c r="C19" t="inlineStr">
@@ -1222,7 +1222,7 @@
       </c>
       <c r="B20" t="inlineStr">
         <is>
-          <t>2026-05-04</t>
+          <t>2026-05-15</t>
         </is>
       </c>
       <c r="C20" t="inlineStr">
@@ -1264,7 +1264,7 @@
       </c>
       <c r="B21" t="inlineStr">
         <is>
-          <t>2026-04-15</t>
+          <t>2026-07-13</t>
         </is>
       </c>
       <c r="C21" t="inlineStr">
@@ -1306,7 +1306,7 @@
       </c>
       <c r="B22" t="inlineStr">
         <is>
-          <t>2026-04-16</t>
+          <t>2026-06-05</t>
         </is>
       </c>
       <c r="C22" t="inlineStr">
@@ -1348,7 +1348,7 @@
       </c>
       <c r="B23" t="inlineStr">
         <is>
-          <t>2026-04-17</t>
+          <t>2026-04-13</t>
         </is>
       </c>
       <c r="C23" t="inlineStr">
@@ -1390,7 +1390,7 @@
       </c>
       <c r="B24" t="inlineStr">
         <is>
-          <t>2026-04-18</t>
+          <t>2026-04-17</t>
         </is>
       </c>
       <c r="C24" t="inlineStr">
@@ -1432,7 +1432,7 @@
       </c>
       <c r="B25" t="inlineStr">
         <is>
-          <t>2026-04-19</t>
+          <t>2026-07-05</t>
         </is>
       </c>
       <c r="C25" t="inlineStr">
@@ -1474,7 +1474,7 @@
       </c>
       <c r="B26" t="inlineStr">
         <is>
-          <t>2026-04-20</t>
+          <t>2026-08-13</t>
         </is>
       </c>
       <c r="C26" t="inlineStr">
@@ -1516,7 +1516,7 @@
       </c>
       <c r="B27" t="inlineStr">
         <is>
-          <t>2026-04-21</t>
+          <t>2026-06-08</t>
         </is>
       </c>
       <c r="C27" t="inlineStr">
@@ -1558,7 +1558,7 @@
       </c>
       <c r="B28" t="inlineStr">
         <is>
-          <t>2026-04-22</t>
+          <t>2026-05-16</t>
         </is>
       </c>
       <c r="C28" t="inlineStr">
@@ -1600,7 +1600,7 @@
       </c>
       <c r="B29" t="inlineStr">
         <is>
-          <t>2026-04-23</t>
+          <t>2026-04-14</t>
         </is>
       </c>
       <c r="C29" t="inlineStr">
@@ -1684,7 +1684,7 @@
       </c>
       <c r="B31" t="inlineStr">
         <is>
-          <t>2026-04-25</t>
+          <t>2026-07-30</t>
         </is>
       </c>
       <c r="C31" t="inlineStr">
@@ -1726,7 +1726,7 @@
       </c>
       <c r="B32" t="inlineStr">
         <is>
-          <t>2026-04-26</t>
+          <t>2026-06-07</t>
         </is>
       </c>
       <c r="C32" t="inlineStr">
@@ -1768,7 +1768,7 @@
       </c>
       <c r="B33" t="inlineStr">
         <is>
-          <t>2026-04-27</t>
+          <t>2026-06-14</t>
         </is>
       </c>
       <c r="C33" t="inlineStr">
@@ -1810,7 +1810,7 @@
       </c>
       <c r="B34" t="inlineStr">
         <is>
-          <t>2026-04-28</t>
+          <t>2026-06-21</t>
         </is>
       </c>
       <c r="C34" t="inlineStr">
@@ -1852,7 +1852,7 @@
       </c>
       <c r="B35" t="inlineStr">
         <is>
-          <t>2026-04-29</t>
+          <t>2026-06-28</t>
         </is>
       </c>
       <c r="C35" t="inlineStr">
@@ -1894,7 +1894,7 @@
       </c>
       <c r="B36" t="inlineStr">
         <is>
-          <t>2026-04-30</t>
+          <t>2026-07-05</t>
         </is>
       </c>
       <c r="C36" t="inlineStr">
@@ -1936,7 +1936,7 @@
       </c>
       <c r="B37" t="inlineStr">
         <is>
-          <t>2026-05-01</t>
+          <t>2026-07-12</t>
         </is>
       </c>
       <c r="C37" t="inlineStr">
@@ -1978,7 +1978,7 @@
       </c>
       <c r="B38" t="inlineStr">
         <is>
-          <t>2026-05-02</t>
+          <t>2026-07-19</t>
         </is>
       </c>
       <c r="C38" t="inlineStr">
@@ -2020,7 +2020,7 @@
       </c>
       <c r="B39" t="inlineStr">
         <is>
-          <t>2026-05-03</t>
+          <t>2026-07-26</t>
         </is>
       </c>
       <c r="C39" t="inlineStr">
@@ -2104,7 +2104,7 @@
       </c>
       <c r="B41" t="inlineStr">
         <is>
-          <t>2026-04-15</t>
+          <t>2026-05-11</t>
         </is>
       </c>
       <c r="C41" t="inlineStr">

</xml_diff>